<commit_message>
docs(release-planning): update planning after J3 and RGPD perturbations
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-28-release-planning-v1.0.xlsx
+++ b/docs/cadrage/equipe-28-release-planning-v1.0.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Downloads\Doc_APOCALIPSSI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IPSSI_25-26\APOCALIPSSI_G28\IPSSI_APOCAL_KIT_GR_28\docs\cadrage\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Garde" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="179">
   <si>
     <t>A</t>
   </si>
@@ -332,9 +332,6 @@
   </si>
   <si>
     <t>Auto-évaluation</t>
-  </si>
-  <si>
-    <t>Commentaire / preuve</t>
   </si>
   <si>
     <t>Les 7 sprints sont planifiés avec jour, horaires et capacité (h-pers) chiffrée</t>
@@ -414,43 +411,10 @@
     <t>Perturbation J2 Technique à 10h00</t>
   </si>
   <si>
-    <t>Développer l’historique F6 et durcir la sécurité face au risque de prompt injection. Ajouter les tests de sécurité nécessaires sans dégrader le flux MVP.</t>
-  </si>
-  <si>
     <t>Finaliser la soumission du quiz, la correction automatique, le score /10 et le détail des bonnes/mauvaises réponses. Stabiliser l’intégration F3–F5.</t>
   </si>
   <si>
     <t>Sprint Review 18h</t>
-  </si>
-  <si>
-    <t>US-06, US-08</t>
-  </si>
-  <si>
-    <t>Perturbation J3 Sécurité à 10h00</t>
-  </si>
-  <si>
-    <t>Finaliser le MVP F1–F6, traiter la conformité RGPD allégée, compléter les pages légales et préparer une démonstration stable de la Release 1.</t>
-  </si>
-  <si>
-    <t>US-09, correctifs MVP, pages légales</t>
-  </si>
-  <si>
-    <t>Perturbation J3-bis RGPD à 14h00 + Release 1 MVP à 17h45</t>
-  </si>
-  <si>
-    <t>Perturbation J4 Livraison/Crise à 10h00</t>
-  </si>
-  <si>
-    <t>US-10, US-11</t>
-  </si>
-  <si>
-    <t>Démarrer la Release 2 avec 2–3 pistes utiles et réalistes. Priorité au tableau de bord enseignant et à la vision des lacunes. Gérer la crise utilisateur J4 avec post-mortem court.</t>
-  </si>
-  <si>
-    <t>Finaliser la Release 2, stabiliser la démo, compléter le post-mortem J4 et préparer les éléments de soutenance.</t>
-  </si>
-  <si>
-    <t>US-12, correctifs R2, post-mortem</t>
   </si>
   <si>
     <t>Release 2 à 17h00</t>
@@ -725,12 +689,149 @@
   <si>
     <t>Hypothèses de planification</t>
   </si>
+  <si>
+    <t>Traiter la perturbation J3 Sécurité : créer un jeu de tests adversariaux, corriger la prompt injection, séparer system prompt et user input, ajouter une validation post-LLM et automatiser au moins un test adversarial dans la CI.</t>
+  </si>
+  <si>
+    <t>US-27, US-28, US-29</t>
+  </si>
+  <si>
+    <t>Perturbation J3 Sécurité à 10h00 · patch sécurité + note sécurité + test CI</t>
+  </si>
+  <si>
+    <t>Traiter la perturbation J3-bis RGPD comme une décision de conformité : enregistrer la demande SAR de Hugo Petit, inventorier les données personnelles, rédiger la réponse écrite, produire une politique de rétention allégée et finaliser la Release 1 MVP.</t>
+  </si>
+  <si>
+    <t>US-30, US-31, US-32, US-33 + correctifs MVP</t>
+  </si>
+  <si>
+    <t>Perturbation J3-bis RGPD · Release 1 MVP à 17h45</t>
+  </si>
+  <si>
+    <t>Démarrer la Release 2 en transformant les décisions RGPD en fonctionnalités : endpoint d’export des données, bouton frontend “Exporter mes données”, et stabilisation des éléments non finalisés en Release 1.</t>
+  </si>
+  <si>
+    <t>US-34, US-35 + éventuels correctifs sécurité/RGPD</t>
+  </si>
+  <si>
+    <t>Perturbation J4 à 10h00 · préparation Release 2</t>
+  </si>
+  <si>
+    <t>Finaliser la Release 2, stabiliser la démo, intégrer les retours sur sécurité/RGPD et préparer le post-mortem J4.</t>
+  </si>
+  <si>
+    <t>Correctifs Release 2 + post-mortem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commentaire </t>
+  </si>
+  <si>
+    <t>Release Planning mis à jour après les perturbations J2, J3 et J3-bis.</t>
+  </si>
+  <si>
+    <t>La priorité reste la livraison du MVP mercredi soir, mais le planning intègre désormais :</t>
+  </si>
+  <si>
+    <r>
+      <t>·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Verdana"/>
+        <family val="2"/>
+      </rPr>
+      <t>la re-estimation de la génération de quiz après benchmark LLM ;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Verdana"/>
+        <family val="2"/>
+      </rPr>
+      <t>le traitement prioritaire de la prompt injection avant la Release 1 ;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Verdana"/>
+        <family val="2"/>
+      </rPr>
+      <t>la prise en compte de la demande RGPD Article 15 de Hugo Petit ;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Verdana"/>
+        <family val="2"/>
+      </rPr>
+      <t>le report des fonctionnalités RGPD plus techniques, comme l’endpoint d’export et le bouton frontend, vers la Release 2 si la capacité ne permet pas leur intégration complète avant mercredi soir.</t>
+    </r>
+  </si>
+  <si>
+    <t>Cette décision permet de sécuriser la Release 1 sans transformer la perturbation RGPD en sprint de code complet.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="28" x14ac:knownFonts="1">
+  <fonts count="29" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -899,6 +1000,13 @@
       <name val="Verdana"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -998,7 +1106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1126,6 +1234,9 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="5"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1158,6 +1269,7 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1478,22 +1590,22 @@
                   <c:v>56</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>56</c:v>
+                  <c:v>61</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>56</c:v>
+                  <c:v>61</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>56</c:v>
+                  <c:v>72</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>56</c:v>
+                  <c:v>82</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>56</c:v>
+                  <c:v>90</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>56</c:v>
+                  <c:v>90</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1635,6 +1747,7 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -2636,7 +2749,7 @@
         <v>9</v>
       </c>
       <c r="C5" s="40" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="86.4" x14ac:dyDescent="0.3">
@@ -2644,7 +2757,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="38" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="2:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2652,7 +2765,7 @@
         <v>11</v>
       </c>
       <c r="C7" s="40" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2660,7 +2773,7 @@
         <v>12</v>
       </c>
       <c r="C8" s="40" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="2:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2668,7 +2781,7 @@
         <v>13</v>
       </c>
       <c r="C9" s="40" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2676,7 +2789,7 @@
         <v>14</v>
       </c>
       <c r="C10" s="40" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.3">
@@ -2691,92 +2804,92 @@
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B16" s="54" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B17" s="52" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B18" s="52" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B19" s="52" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B20" s="53" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
     </row>
     <row r="21" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B21" s="53" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B22" s="53" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
     </row>
     <row r="23" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B23" s="52" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B24" s="53" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B25" s="53" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
     </row>
     <row r="26" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B26" s="53" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B27" s="53" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B28" s="53" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
     </row>
     <row r="29" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B29" s="53" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
     </row>
     <row r="30" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B30" s="52" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
     </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B31" s="52" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
     </row>
     <row r="32" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B32" s="52" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B33" s="52" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -2883,13 +2996,13 @@
         <v>38</v>
       </c>
       <c r="F10" s="44" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G10" s="16" t="s">
         <v>38</v>
       </c>
       <c r="H10" s="16" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="69" x14ac:dyDescent="0.3">
@@ -2909,13 +3022,13 @@
         <v>42</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G11" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="H11" s="19" t="s">
         <v>122</v>
-      </c>
-      <c r="H11" s="19" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -2935,13 +3048,13 @@
         <v>46</v>
       </c>
       <c r="F12" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="G12" s="22" t="s">
         <v>125</v>
       </c>
-      <c r="G12" s="22" t="s">
+      <c r="H12" s="22" t="s">
         <v>126</v>
-      </c>
-      <c r="H12" s="22" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
@@ -2961,16 +3074,16 @@
         <v>42</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="G13" s="45" t="s">
         <v>49</v>
       </c>
       <c r="H13" s="45" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A14" s="21" t="s">
         <v>50</v>
       </c>
@@ -2987,16 +3100,16 @@
         <v>46</v>
       </c>
       <c r="F14" s="46" t="s">
-        <v>128</v>
+        <v>160</v>
       </c>
       <c r="G14" s="46" t="s">
-        <v>131</v>
+        <v>161</v>
       </c>
       <c r="H14" s="46" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A15" s="24" t="s">
         <v>52</v>
       </c>
@@ -3013,16 +3126,16 @@
         <v>46</v>
       </c>
       <c r="F15" s="47" t="s">
-        <v>133</v>
+        <v>163</v>
       </c>
       <c r="G15" s="47" t="s">
-        <v>134</v>
+        <v>164</v>
       </c>
       <c r="H15" s="47" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
         <v>54</v>
       </c>
@@ -3039,13 +3152,13 @@
         <v>56</v>
       </c>
       <c r="F16" s="46" t="s">
-        <v>138</v>
+        <v>166</v>
       </c>
       <c r="G16" s="46" t="s">
-        <v>137</v>
+        <v>167</v>
       </c>
       <c r="H16" s="46" t="s">
-        <v>136</v>
+        <v>168</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -3065,13 +3178,13 @@
         <v>60</v>
       </c>
       <c r="F17" s="47" t="s">
-        <v>139</v>
+        <v>169</v>
       </c>
       <c r="G17" s="47" t="s">
-        <v>140</v>
+        <v>170</v>
       </c>
       <c r="H17" s="47" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -3091,13 +3204,13 @@
         <v>38</v>
       </c>
       <c r="F18" s="48" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="G18" s="28" t="s">
         <v>38</v>
       </c>
       <c r="H18" s="48" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
@@ -3163,7 +3276,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -3269,7 +3382,7 @@
       </c>
       <c r="D11" s="49"/>
       <c r="E11" s="51">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3284,7 +3397,7 @@
       </c>
       <c r="D12" s="49"/>
       <c r="E12" s="51">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3299,7 +3412,7 @@
       </c>
       <c r="D13" s="49"/>
       <c r="E13" s="51">
-        <v>56</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3314,7 +3427,7 @@
       </c>
       <c r="D14" s="49"/>
       <c r="E14" s="51">
-        <v>56</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3329,7 +3442,7 @@
       </c>
       <c r="D15" s="49"/>
       <c r="E15" s="51">
-        <v>56</v>
+        <v>90</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3344,7 +3457,7 @@
       </c>
       <c r="D16" s="49"/>
       <c r="E16" s="51">
-        <v>56</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -3358,9 +3471,53 @@
         <v>98</v>
       </c>
     </row>
+    <row r="37" spans="2:2" ht="16.2" x14ac:dyDescent="0.3">
+      <c r="B37" s="55" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2" ht="16.2" x14ac:dyDescent="0.3">
+      <c r="B38" s="55"/>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B39" s="52" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B40" s="52" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="41" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B41" s="53" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="42" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B42" s="53" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="43" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B43" s="53" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="44" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B44" s="53" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="45" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B45" s="52" t="s">
+        <v>178</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -3393,107 +3550,107 @@
       <c r="C5" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="D5" t="s">
-        <v>103</v>
+      <c r="D5" s="14" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="36" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="D6" s="36" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C7" s="37" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="D7" s="36" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="36" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="D8" s="36" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="36" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="D9" s="36" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="36" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="D10" s="36" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="36" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="D11" s="36" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="36" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="D12" s="36" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="36" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C13" s="37" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="D13" s="36" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="36" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C14" s="37" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D14" s="36" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>